<commit_message>
Give Chen a dual US/HK footprint so FBAR fires on the $2M HK aggregate.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/demo_docs/chen_trust.xlsx
+++ b/demo_docs/chen_trust.xlsx
@@ -9,8 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Holdings" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Dividends" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Foreign accounts" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Dividends" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Notes" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
   <si>
     <t xml:space="preserve">Holding</t>
   </si>
@@ -39,7 +40,7 @@
     <t xml:space="preserve">Ownership</t>
   </si>
   <si>
-    <t xml:space="preserve">Northline Inc. (NASDAQ-listed, founded by settlor ~20 years ago)</t>
+    <t xml:space="preserve">Northline Inc. (NYSE-listed, founded by settlor ~20 years ago)</t>
   </si>
   <si>
     <t xml:space="preserve">public company shares</t>
@@ -51,6 +52,33 @@
     <t xml:space="preserve">cash</t>
   </si>
   <si>
+    <t xml:space="preserve">Institution / account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max balance USD (year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSBC Hong Kong bank account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hong Kong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HK brokerage custody account</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brokerage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aggregate maximum</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quarter 2026</t>
   </si>
   <si>
@@ -84,7 +112,13 @@
     <t xml:space="preserve">The Chen Family Trust is a US family trust with Massachusetts situs. The trust is a US person.</t>
   </si>
   <si>
-    <t xml:space="preserve">The settlor founded Northline Inc. and took it public about 20 years ago; the trust still owns 8 percent of the listed shares.</t>
+    <t xml:space="preserve">The settlor founded Northline Inc. and took it public on the NYSE about 20 years ago; the trust still owns 8 percent of the listed shares.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Northline Inc. operates in the US, mainland China, Hong Kong, and the EU through local subsidiaries.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr. Chen and his family moved to Hong Kong 10 years ago (2016); he is a US person and a Hong Kong resident.</t>
   </si>
   <si>
     <t xml:space="preserve">Dividends are paid to the trust each year and partly distributed to beneficiaries.</t>
@@ -603,11 +637,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
   </cols>
@@ -617,84 +651,52 @@
         <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>9600000</v>
+      <c r="C2" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="D2" s="3" t="n">
-        <f aca="false">B2*C2</f>
-        <v>2112000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="2" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>9600000</v>
-      </c>
       <c r="D3" s="3" t="n">
-        <f aca="false">B3*C3</f>
-        <v>2112000</v>
+        <v>1750000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>9600000</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <f aca="false">B4*C4</f>
-        <v>2208000</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>9600000</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <f aca="false">B5*C5</f>
-        <v>2208000</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6" t="n">
-        <f aca="false">SUM(D2:D5)</f>
-        <v>8640000</v>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="6" t="n">
+        <f aca="false">SUM(D2:D3)</f>
+        <v>2000000</v>
       </c>
     </row>
   </sheetData>
@@ -713,7 +715,117 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>9600000</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <f aca="false">B2*C2</f>
+        <v>2112000</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>9600000</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <f aca="false">B3*C3</f>
+        <v>2112000</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>9600000</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <f aca="false">B4*C4</f>
+        <v>2208000</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>9600000</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <f aca="false">B5*C5</f>
+        <v>2208000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="5"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6" t="n">
+        <f aca="false">SUM(D2:D5)</f>
+        <v>8640000</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -721,32 +833,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>21</v>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>22</v>
+      <c r="A7" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>23</v>
+      <c r="A9" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>